<commit_message>
change import in check and run
</commit_message>
<xml_diff>
--- a/score_correct_Transformer_median.xlsx
+++ b/score_correct_Transformer_median.xlsx
@@ -759,7 +759,7 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -773,7 +773,7 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -787,7 +787,7 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="26">
@@ -2341,7 +2341,7 @@
         <v>1</v>
       </c>
       <c r="D136" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -2355,7 +2355,7 @@
         <v>1</v>
       </c>
       <c r="D137" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -2369,7 +2369,7 @@
         <v>1</v>
       </c>
       <c r="D138" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -2831,7 +2831,7 @@
         <v>1</v>
       </c>
       <c r="D171" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="172">

</xml_diff>